<commit_message>
Classeur de campagne : feuille Comparaison (hériter, gagner ou placer 300 000 € ; prix du logement)
Toutes les valeurs sont des formules (barème des successions, impôt sur le
revenu 2026, CSG, PFU), montant modifiable, avec contrôle d'écart nul par
rapport au site.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188qNw1StBQkFA1rFcQwdyx
</commit_message>
<xml_diff>
--- a/campagne/chiffrages/Chiffrage_Campagne.xlsx
+++ b/campagne/chiffrages/Chiffrage_Campagne.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Calage" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Tranches" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Résultats" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Sources" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Comparaison" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Sources" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -70,8 +71,78 @@
 </comments>
 </file>
 
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="B7" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">CGI, art. 779</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Vieillesse 7,30 % + Agirc-Arrco et CEG 4,01 % ; non comptées dans le prélèvement, car elles ouvrent des droits</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">9,2 % + 0,5 %, × 98,25 %</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">6,8 %, × 98,25 %</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B30" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">12,8 % d'impôt + 18,6 % de prélèvements sociaux</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="149">
   <si>
     <t xml:space="preserve">Chiffrage du site « L'héritage, ça se décide »</t>
   </si>
@@ -94,6 +165,9 @@
     <t xml:space="preserve">Résultats : recettes de 2025 à 2040, qui suivent le flux successoral, plus les plus-values latentes.</t>
   </si>
   <si>
+    <t xml:space="preserve">Comparaison : ce que coûte la même somme reçue en héritage, gagnée en salaire ou touchée en dividendes ; hausse des prix du logement depuis 2000.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vérification</t>
   </si>
   <si>
@@ -361,6 +435,99 @@
     <t xml:space="preserve">Écart classeur − site (doit être nul)</t>
   </si>
   <si>
+    <t xml:space="preserve">Hériter, gagner ou placer la même somme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barèmes 2026, personne seule. Modifiez le montant en B4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montant reçu (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. En héritage d'un parent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abattement (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Droits de succession (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème en ligne directe (CGI, art. 777), feuille Tranches, colonnes R et S.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. En salaire brut, sur plusieurs années</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre d'années</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cotisations salariales hors CSG (déductibles)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSG et CRDS (sur 98,25 % du brut)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dont CSG déductible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abattement pour frais professionnels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salaire brut annuel (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenu imposable annuel (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème de l'impôt sur le revenu 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impôt sur le revenu annuel (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSG et CRDS annuelles (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSG, CRDS et impôt sur le revenu, sur la période (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. En dividendes ou intérêts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prélèvement forfaitaire unique 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prélèvement (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrôle : héritage, salaire, dividendes du site pour 300 000 € (écart en colonne C, doit être nul)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logement : prix des logements anciens depuis 2000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indice 1er trimestre 2000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insee, série 010567059 (base 100 en 2015, CVS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indice 4e trimestre 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prix à la consommation 2000 ; 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eurostat, IPCH France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausse des prix</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sources</t>
   </si>
   <si>
@@ -398,13 +565,37 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.legifrance.gouv.fr/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème de l'impôt sur le revenu 2026, PFU 31,4 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loi de finances pour 2026 ; LFSS 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prix des logements anciens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insee, série 010567059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.insee.fr/fr/statistiques/serie/010567059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prix à la consommation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eurostat, IPCH (prc_hicp_aind)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ec.europa.eu/eurostat/databrowser/view/prc_hicp_aind/default/table</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; €&quot;;\-#,##0&quot; €&quot;;\-"/>
     <numFmt numFmtId="166" formatCode="0.0%;\-0.0%;\-"/>
@@ -414,6 +605,7 @@
     <numFmt numFmtId="170" formatCode="#,##0.00&quot; Md€&quot;;\-#,##0.00&quot; Md€&quot;;\-"/>
     <numFmt numFmtId="171" formatCode="0"/>
     <numFmt numFmtId="172" formatCode="#,##0.0&quot; Md€&quot;;\-#,##0.0&quot; Md€&quot;;\-"/>
+    <numFmt numFmtId="173" formatCode="0.00%;\-0.00%;\-"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -571,7 +763,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -681,6 +873,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -940,7 +1148,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -982,58 +1190,63 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="8" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1063,28 +1276,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" s="11" t="n">
         <v>200000</v>
@@ -1095,7 +1308,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>800000</v>
@@ -1106,7 +1319,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" s="11" t="n">
         <v>1200000</v>
@@ -1117,7 +1330,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>2000000</v>
@@ -1128,7 +1341,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="11" t="n">
         <v>4000000</v>
@@ -1139,7 +1352,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B10" s="11" t="n">
         <v>6000000</v>
@@ -1150,7 +1363,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>1000000000000000</v>
@@ -1159,12 +1372,12 @@
         <v>0.5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>0</v>
@@ -1172,18 +1385,18 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" s="13" t="n">
         <v>1</v>
@@ -1192,7 +1405,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B17" s="13" t="n">
         <v>1</v>
@@ -1201,18 +1414,18 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B18" s="13" t="n">
         <v>0.333333333333333</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B19" s="13" t="n">
         <v>1</v>
@@ -1221,13 +1434,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1256,17 +1469,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4" s="14" t="n">
         <v>15</v>
@@ -1274,7 +1487,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B4*1000000000/SUMPRODUCT(Tranches!$B$6:$B$19,Tranches!$F$6:$F$19)</f>
@@ -1283,7 +1496,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6" s="16" t="n">
         <f aca="false">B5*SUMPRODUCT(Tranches!$B$6:$B$19,Tranches!$D$6:$D$19)/1000000000</f>
@@ -1292,7 +1505,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>0.6</v>
@@ -1300,7 +1513,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" s="13" t="n">
         <v>0.5472653720394</v>
@@ -1308,7 +1521,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="13" t="n">
         <v>0.70145161245459</v>
@@ -1316,7 +1529,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11" s="13" t="n">
         <v>0.787510407002557</v>
@@ -1324,7 +1537,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" s="11" t="n">
         <v>100000</v>
@@ -1363,64 +1576,64 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q4" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="R5" s="17" t="n">
         <v>8072</v>
@@ -1431,7 +1644,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0.1</v>
@@ -1495,7 +1708,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>0.1</v>
@@ -1559,7 +1772,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>0.1</v>
@@ -1623,7 +1836,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B9" s="18" t="n">
         <v>0.1</v>
@@ -1687,7 +1900,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>0.1</v>
@@ -1751,7 +1964,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B11" s="18" t="n">
         <v>0.1</v>
@@ -1815,7 +2028,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>0.1</v>
@@ -1873,7 +2086,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B13" s="18" t="n">
         <v>0.1</v>
@@ -1931,7 +2144,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B14" s="18" t="n">
         <v>0.1</v>
@@ -1989,7 +2202,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B15" s="18" t="n">
         <v>0.05</v>
@@ -2047,7 +2260,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B16" s="18" t="n">
         <v>0.04</v>
@@ -2105,7 +2318,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B17" s="18" t="n">
         <v>0.005</v>
@@ -2163,7 +2376,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B18" s="18" t="n">
         <v>0.004</v>
@@ -2221,7 +2434,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B19" s="18" t="n">
         <v>0.001</v>
@@ -2302,12 +2515,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D3" s="21" t="n">
         <f aca="false">Calage!$B$5*SUMPRODUCT(Tranches!$B$6:$B$19,Tranches!$N$6:$N$19)/1000000000</f>
@@ -2316,7 +2529,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D4" s="21" t="n">
         <f aca="false">Calage!$B$5*SUMPRODUCT(Tranches!$B$6:$B$19,Tranches!$O$6:$O$19)/1000000000</f>
@@ -2325,25 +2538,25 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2780,7 +2993,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F24" s="25" t="n">
         <f aca="false">SUM(F7:F22)</f>
@@ -2789,7 +3002,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F26" s="27" t="n">
         <v>23.9385</v>
@@ -2797,7 +3010,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F27" s="21" t="n">
         <f aca="false">ROUND(F7-F26,2)</f>
@@ -2820,7 +3033,351 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D42"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B8" s="28" t="n">
+        <f aca="false">MAX(0,MIN(MAX(0,$B$4-$B$7),Tranches!$R$5)-0)*Tranches!$S$5+MAX(0,MIN(MAX(0,$B$4-$B$7),Tranches!$R$6)-Tranches!$R$5)*Tranches!$S$6+MAX(0,MIN(MAX(0,$B$4-$B$7),Tranches!$R$7)-Tranches!$R$6)*Tranches!$S$7+MAX(0,MIN(MAX(0,$B$4-$B$7),Tranches!$R$8)-Tranches!$R$7)*Tranches!$S$8+MAX(0,MIN(MAX(0,$B$4-$B$7),Tranches!$R$9)-Tranches!$R$8)*Tranches!$S$9+MAX(0,MIN(MAX(0,$B$4-$B$7),Tranches!$R$10)-Tranches!$R$9)*Tranches!$S$10+MAX(0,MIN(MAX(0,$B$4-$B$7),Tranches!$R$11)-Tranches!$R$10)*Tranches!$S$11</f>
+        <v>38194.35</v>
+      </c>
+      <c r="C8" s="20" t="n">
+        <f aca="false">B8/$B$4</f>
+        <v>0.1273145</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" s="29" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" s="30" t="n">
+        <v>0.1131</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="30" t="n">
+        <v>0.0953025</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="30" t="n">
+        <v>0.06681</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="19" t="n">
+        <f aca="false">B4/B11</f>
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" s="19" t="n">
+        <f aca="false">B16*(1-B12-B14)*(1-B15)</f>
+        <v>44284.86</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>11600</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>29579</v>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>84577</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>181917</v>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>1000000000000000</v>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="19" t="n">
+        <f aca="false">MAX(0,MIN(B17,$B$19)-0)*$C$19+MAX(0,MIN(B17,$B$20)-$B$19)*$C$20+MAX(0,MIN(B17,$B$21)-$B$20)*$C$21+MAX(0,MIN(B17,$B$22)-$B$21)*$C$22+MAX(0,MIN(B17,$B$23)-$B$22)*$C$23</f>
+        <v>6389.448</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B26" s="19" t="n">
+        <f aca="false">B16*B13</f>
+        <v>5718.15</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B27" s="28" t="n">
+        <f aca="false">B11*(B25+B26)</f>
+        <v>60537.99</v>
+      </c>
+      <c r="C27" s="20" t="n">
+        <f aca="false">B27/$B$4</f>
+        <v>0.2017933</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B30" s="12" t="n">
+        <v>0.314</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B31" s="28" t="n">
+        <f aca="false">B4*B30</f>
+        <v>94200</v>
+      </c>
+      <c r="C31" s="20" t="n">
+        <f aca="false">B31/$B$4</f>
+        <v>0.314</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B33" s="17" t="n">
+        <v>38194.35</v>
+      </c>
+      <c r="C33" s="15" t="n">
+        <f aca="false">IF($B$4=300000,ROUND(B8-B33,0),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="17" t="n">
+        <v>60537.99</v>
+      </c>
+      <c r="C34" s="15" t="n">
+        <f aca="false">IF($B$4=300000,ROUND(B27-B34,0),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="17" t="n">
+        <v>94200</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <f aca="false">IF($B$4=300000,ROUND(B31-B35,0),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B38" s="26" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B39" s="26" t="n">
+        <v>127.3</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B40" s="31" t="n">
+        <f aca="false">B39/B38-1</f>
+        <v>1.66317991631799</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B41" s="26" t="n">
+        <v>78.23</v>
+      </c>
+      <c r="C41" s="26" t="n">
+        <v>124.43</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B42" s="31" t="n">
+        <f aca="false">C41/B41-1</f>
+        <v>0.59056627892113</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -2830,51 +3387,84 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>97</v>
+        <v>129</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>98</v>
+        <v>130</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>99</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>102</v>
+        <v>133</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>103</v>
+        <v>135</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>105</v>
+        <v>136</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>108</v>
+        <v>139</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2882,6 +3472,9 @@
     <hyperlink ref="C4" r:id="rId1" display="https://www.cae-eco.fr/repenser-lheritage"/>
     <hyperlink ref="C5" r:id="rId2" display="https://www.jean-jaures.org/publication/face-a-la-grande-transmission-limpot-sur-les-grandes-successions/"/>
     <hyperlink ref="C6" r:id="rId3" display="https://www.legifrance.gouv.fr/"/>
+    <hyperlink ref="C7" r:id="rId4" display="https://www.legifrance.gouv.fr/"/>
+    <hyperlink ref="C8" r:id="rId5" display="https://www.insee.fr/fr/statistiques/serie/010567059"/>
+    <hyperlink ref="C9" r:id="rId6" display="https://ec.europa.eu/eurostat/databrowser/view/prc_hicp_aind/default/table"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>